<commit_message>
clean up master branch and make similar to CRAN package
</commit_message>
<xml_diff>
--- a/inst/extdata/example_BioPlex_plate1.xlsx
+++ b/inst/extdata/example_BioPlex_plate1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11124"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/argyropoulos.d/Documents/GitHub/pvserotat/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dionne/Documents/GitHub/SeroTrackR/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B9F53E-BDA7-7444-8CC2-EB6F1558F22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686BBC0F-95F1-184E-9794-290A873EC0DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45000" yWindow="-5880" windowWidth="22760" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45000" yWindow="-5200" windowWidth="22760" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bioplex_example" sheetId="1" r:id="rId1"/>

</xml_diff>